<commit_message>
Update master_schedule.xlsx and app.css for new styles and schedule changes
</commit_message>
<xml_diff>
--- a/storage/app/master_schedule.xlsx
+++ b/storage/app/master_schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Laravel Projects\lecturer-invigilation-portal\storage\app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CC90C04-AF19-48DD-B685-A484CC5592A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F767CEB5-7019-43BE-917A-548DA4677275}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="192">
   <si>
     <t>DATE</t>
   </si>
@@ -391,9 +391,6 @@
     <t>Mr. Dancan Eric Ogonji</t>
   </si>
   <si>
-    <t>Brian Mweu</t>
-  </si>
-  <si>
     <t>Dr Watson Kanuku</t>
   </si>
   <si>
@@ -466,18 +463,12 @@
     <t>ACS 323A</t>
   </si>
   <si>
-    <t>ACS 102A</t>
-  </si>
-  <si>
     <t>ACS 101T</t>
   </si>
   <si>
     <t>ACS 100T</t>
   </si>
   <si>
-    <t>DICT 111A</t>
-  </si>
-  <si>
     <t>DICT 111T</t>
   </si>
   <si>
@@ -614,6 +605,9 @@
   </si>
   <si>
     <t>ACS331B/MIS 228B</t>
+  </si>
+  <si>
+    <t>DICT 111A/ACS102A</t>
   </si>
 </sst>
 </file>
@@ -1347,7 +1341,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G131"/>
+  <dimension ref="A1:G130"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.81640625" style="2" customWidth="1"/>
@@ -1407,7 +1401,7 @@
     <row r="7" spans="1:7" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A7" s="1"/>
       <c r="B7" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C7" s="4"/>
       <c r="D7" s="7"/>
@@ -1475,10 +1469,10 @@
         <v>17</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>29</v>
@@ -1494,7 +1488,7 @@
       <c r="A13" s="53"/>
       <c r="B13" s="19"/>
       <c r="C13" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D13" s="13">
         <v>35</v>
@@ -1513,7 +1507,7 @@
       <c r="A14" s="53"/>
       <c r="B14" s="19"/>
       <c r="C14" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D14" s="13">
         <v>35</v>
@@ -1562,7 +1556,7 @@
       <c r="A17" s="53"/>
       <c r="B17" s="19"/>
       <c r="C17" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D17" s="21">
         <v>12</v>
@@ -1581,7 +1575,7 @@
       <c r="A18" s="53"/>
       <c r="B18" s="19"/>
       <c r="C18" s="11" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D18" s="21">
         <v>58</v>
@@ -1600,7 +1594,7 @@
       <c r="A19" s="42"/>
       <c r="B19" s="19"/>
       <c r="C19" s="11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D19" s="21">
         <v>40</v>
@@ -1657,7 +1651,7 @@
         <v>70</v>
       </c>
       <c r="G22" s="18" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -1702,7 +1696,7 @@
       <c r="A25" s="53"/>
       <c r="B25" s="55"/>
       <c r="C25" s="39" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D25" s="17">
         <v>42</v>
@@ -1732,7 +1726,7 @@
         <v>11</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D27" s="13">
         <v>19</v>
@@ -1751,7 +1745,7 @@
       <c r="A28" s="53"/>
       <c r="B28" s="56"/>
       <c r="C28" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D28" s="13">
         <v>42</v>
@@ -1878,7 +1872,7 @@
       <c r="A35" s="57"/>
       <c r="B35" s="22"/>
       <c r="C35" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D35" s="21">
         <v>42</v>
@@ -1930,7 +1924,7 @@
         <v>14</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D39" s="23">
         <v>20</v>
@@ -1949,7 +1943,7 @@
       <c r="A40" s="57"/>
       <c r="B40" s="25"/>
       <c r="C40" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D40" s="23">
         <v>44</v>
@@ -1981,13 +1975,13 @@
         <v>7</v>
       </c>
       <c r="C42" s="11" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="D42" s="13" t="s">
         <v>105</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="F42" s="9" t="s">
         <v>77</v>
@@ -2000,7 +1994,7 @@
       <c r="A43" s="52"/>
       <c r="B43" s="22"/>
       <c r="C43" s="11" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="D43" s="13" t="s">
         <v>117</v>
@@ -2019,7 +2013,7 @@
       <c r="A44" s="52"/>
       <c r="B44" s="26"/>
       <c r="C44" s="11" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D44" s="13">
         <v>16</v>
@@ -2038,7 +2032,7 @@
       <c r="A45" s="52"/>
       <c r="B45" s="26"/>
       <c r="C45" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D45" s="13">
         <v>45</v>
@@ -2068,7 +2062,7 @@
         <v>10</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D47" s="23">
         <v>21</v>
@@ -2087,7 +2081,7 @@
       <c r="A48" s="52"/>
       <c r="B48" s="27"/>
       <c r="C48" s="9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D48" s="23">
         <v>50</v>
@@ -2106,7 +2100,7 @@
       <c r="A49" s="52"/>
       <c r="B49" s="27"/>
       <c r="C49" s="9" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D49" s="23">
         <v>25</v>
@@ -2182,16 +2176,16 @@
         <v>16</v>
       </c>
       <c r="C55" s="9" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="D55" s="17" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="E55" s="11" t="s">
         <v>29</v>
       </c>
       <c r="F55" s="14" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="G55" s="18" t="s">
         <v>73</v>
@@ -2201,7 +2195,7 @@
       <c r="A56" s="52"/>
       <c r="B56" s="28"/>
       <c r="C56" s="43" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D56" s="17">
         <v>33</v>
@@ -2231,7 +2225,7 @@
         <v>15</v>
       </c>
       <c r="C58" s="11" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="D58" s="23" t="s">
         <v>116</v>
@@ -2250,7 +2244,7 @@
       <c r="A59" s="52"/>
       <c r="B59" s="30"/>
       <c r="C59" s="9" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D59" s="21" t="s">
         <v>117</v>
@@ -2269,1242 +2263,1223 @@
       <c r="A60" s="52"/>
       <c r="B60" s="30"/>
       <c r="C60" s="9" t="s">
-        <v>144</v>
+        <v>45</v>
       </c>
       <c r="D60" s="21">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F60" s="9" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="G60" s="14" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" s="52"/>
       <c r="B61" s="30"/>
       <c r="C61" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D61" s="21">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="E61" s="11" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F61" s="9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G61" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62" s="52"/>
       <c r="B62" s="30"/>
       <c r="C62" s="9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D62" s="21">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="F62" s="9" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="G62" s="14" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63" s="52"/>
       <c r="B63" s="30"/>
       <c r="C63" s="9" t="s">
-        <v>44</v>
+        <v>143</v>
       </c>
       <c r="D63" s="21">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E63" s="11" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="F63" s="9" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="G63" s="14" t="s">
-        <v>100</v>
+        <v>83</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="52"/>
       <c r="B64" s="30"/>
       <c r="C64" s="9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D64" s="21">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E64" s="11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F64" s="9" t="s">
-        <v>83</v>
+        <v>106</v>
       </c>
       <c r="G64" s="14" t="s">
-        <v>83</v>
+        <v>106</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="52"/>
       <c r="B65" s="30"/>
       <c r="C65" s="9" t="s">
-        <v>146</v>
+        <v>191</v>
       </c>
       <c r="D65" s="21">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="E65" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F65" s="9" t="s">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="G65" s="14" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="66" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="52"/>
       <c r="B66" s="30"/>
       <c r="C66" s="9" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D66" s="21">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="E66" s="11" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="F66" s="9" t="s">
-        <v>119</v>
+        <v>75</v>
       </c>
       <c r="G66" s="14" t="s">
-        <v>109</v>
+        <v>75</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="52"/>
       <c r="B67" s="30"/>
       <c r="C67" s="9" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D67" s="21">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="E67" s="11" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="F67" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G67" s="14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="52"/>
       <c r="B68" s="30"/>
       <c r="C68" s="9" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D68" s="21">
-        <v>17</v>
+        <v>52</v>
       </c>
       <c r="E68" s="11" t="s">
-        <v>54</v>
+        <v>122</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="G68" s="14" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="69" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="52"/>
       <c r="B69" s="30"/>
       <c r="C69" s="9" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D69" s="21">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="E69" s="11" t="s">
-        <v>123</v>
+        <v>42</v>
       </c>
       <c r="F69" s="9" t="s">
-        <v>83</v>
+        <v>106</v>
       </c>
       <c r="G69" s="14" t="s">
-        <v>71</v>
+        <v>106</v>
       </c>
     </row>
     <row r="70" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="52"/>
       <c r="B70" s="30"/>
       <c r="C70" s="9" t="s">
-        <v>151</v>
+        <v>180</v>
       </c>
       <c r="D70" s="21">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="E70" s="11" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="F70" s="9" t="s">
-        <v>106</v>
+        <v>75</v>
       </c>
       <c r="G70" s="14" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="52"/>
-      <c r="B71" s="30"/>
-      <c r="C71" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="D71" s="21">
-        <v>25</v>
-      </c>
-      <c r="E71" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="F71" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="G71" s="14" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B71" s="44"/>
+      <c r="C71" s="44"/>
+      <c r="D71" s="44"/>
+      <c r="E71" s="44"/>
+      <c r="F71" s="44"/>
+      <c r="G71" s="44"/>
+    </row>
+    <row r="72" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="52"/>
-      <c r="B72" s="44"/>
-      <c r="C72" s="44"/>
-      <c r="D72" s="44"/>
-      <c r="E72" s="44"/>
-      <c r="F72" s="44"/>
-      <c r="G72" s="44"/>
+      <c r="B72" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="C72" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="D72" s="17">
+        <v>13</v>
+      </c>
+      <c r="E72" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="F72" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="G72" s="18" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="73" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="52"/>
-      <c r="B73" s="22" t="s">
-        <v>14</v>
-      </c>
-      <c r="C73" s="9" t="s">
-        <v>152</v>
-      </c>
-      <c r="D73" s="17">
-        <v>13</v>
-      </c>
-      <c r="E73" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="F73" s="18" t="s">
-        <v>100</v>
-      </c>
-      <c r="G73" s="18" t="s">
-        <v>100</v>
+      <c r="B73" s="22"/>
+      <c r="C73" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="D73" s="23">
+        <v>15</v>
+      </c>
+      <c r="E73" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F73" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="G73" s="14" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="74" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="52"/>
       <c r="B74" s="22"/>
       <c r="C74" s="11" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D74" s="23">
-        <v>15</v>
+        <v>57</v>
       </c>
       <c r="E74" s="9" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="F74" s="14" t="s">
         <v>74</v>
       </c>
       <c r="G74" s="14" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
     </row>
     <row r="75" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="52"/>
       <c r="B75" s="22"/>
       <c r="C75" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="D75" s="23">
-        <v>57</v>
-      </c>
-      <c r="E75" s="9" t="s">
-        <v>38</v>
+        <v>55</v>
+      </c>
+      <c r="D75" s="23" t="s">
+        <v>115</v>
+      </c>
+      <c r="E75" s="11" t="s">
+        <v>39</v>
       </c>
       <c r="F75" s="14" t="s">
-        <v>74</v>
+        <v>109</v>
       </c>
       <c r="G75" s="14" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="76" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="52"/>
-      <c r="B76" s="22"/>
-      <c r="C76" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="D76" s="23" t="s">
-        <v>115</v>
-      </c>
-      <c r="E76" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="F76" s="14" t="s">
-        <v>109</v>
-      </c>
-      <c r="G76" s="14" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="77" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B76" s="44"/>
+      <c r="C76" s="44"/>
+      <c r="D76" s="44"/>
+      <c r="E76" s="44"/>
+      <c r="F76" s="44"/>
+      <c r="G76" s="31"/>
+    </row>
+    <row r="77" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="52"/>
-      <c r="B77" s="44"/>
-      <c r="C77" s="44"/>
-      <c r="D77" s="44"/>
-      <c r="E77" s="44"/>
-      <c r="F77" s="44"/>
-      <c r="G77" s="31"/>
+      <c r="B77" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="C77" s="41" t="s">
+        <v>112</v>
+      </c>
+      <c r="D77" s="23">
+        <v>33</v>
+      </c>
+      <c r="E77" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="F77" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="G77" s="14" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="78" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="52"/>
-      <c r="B78" s="22" t="s">
-        <v>13</v>
-      </c>
+      <c r="B78" s="32"/>
       <c r="C78" s="41" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D78" s="23">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="E78" s="11" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F78" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="G78" s="14" t="s">
+      <c r="G78" s="9" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="79" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A79" s="52"/>
-      <c r="B79" s="32"/>
-      <c r="C79" s="41" t="s">
-        <v>113</v>
-      </c>
-      <c r="D79" s="23">
-        <v>45</v>
-      </c>
-      <c r="E79" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="F79" s="14" t="s">
-        <v>114</v>
-      </c>
-      <c r="G79" s="9" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="33"/>
-      <c r="B80" s="44"/>
-      <c r="C80" s="44"/>
-      <c r="D80" s="44"/>
-      <c r="E80" s="44"/>
-      <c r="F80" s="44"/>
-      <c r="G80" s="44"/>
+    <row r="79" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="33"/>
+      <c r="B79" s="44"/>
+      <c r="C79" s="44"/>
+      <c r="D79" s="44"/>
+      <c r="E79" s="44"/>
+      <c r="F79" s="44"/>
+      <c r="G79" s="44"/>
+    </row>
+    <row r="80" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A80" s="52" t="s">
+        <v>188</v>
+      </c>
+      <c r="B80" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="C80" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="D80" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="E80" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="F80" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="G80" s="18" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="81" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A81" s="52" t="s">
-        <v>191</v>
-      </c>
-      <c r="B81" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="C81" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="D81" s="17" t="s">
-        <v>72</v>
+      <c r="A81" s="52"/>
+      <c r="B81" s="42"/>
+      <c r="C81" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="D81" s="17">
+        <v>12</v>
       </c>
       <c r="E81" s="11" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="F81" s="18" t="s">
-        <v>73</v>
-      </c>
-      <c r="G81" s="18" t="s">
-        <v>73</v>
+        <v>70</v>
+      </c>
+      <c r="G81" s="14" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="82" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="52"/>
       <c r="B82" s="42"/>
       <c r="C82" s="18" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D82" s="17">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="E82" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="F82" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="G82" s="18" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="52"/>
+      <c r="B83" s="44"/>
+      <c r="C83" s="44"/>
+      <c r="D83" s="44"/>
+      <c r="E83" s="44"/>
+      <c r="F83" s="44"/>
+      <c r="G83" s="44"/>
+    </row>
+    <row r="84" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A84" s="52"/>
+      <c r="B84" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="C84" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="D84" s="13">
+        <v>17</v>
+      </c>
+      <c r="E84" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="F82" s="18" t="s">
-        <v>70</v>
-      </c>
-      <c r="G82" s="14" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A83" s="52"/>
-      <c r="B83" s="42"/>
-      <c r="C83" s="18" t="s">
-        <v>156</v>
-      </c>
-      <c r="D83" s="17">
-        <v>49</v>
-      </c>
-      <c r="E83" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="F83" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="G83" s="18" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="52"/>
-      <c r="B84" s="44"/>
-      <c r="C84" s="44"/>
-      <c r="D84" s="44"/>
-      <c r="E84" s="44"/>
-      <c r="F84" s="44"/>
-      <c r="G84" s="44"/>
+      <c r="F84" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="G84" s="14" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="85" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="52"/>
-      <c r="B85" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="C85" s="18" t="s">
-        <v>157</v>
+      <c r="B85" s="22"/>
+      <c r="C85" s="14" t="s">
+        <v>155</v>
       </c>
       <c r="D85" s="13">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="E85" s="11" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="F85" s="9" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="G85" s="14" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="52"/>
-      <c r="B86" s="22"/>
-      <c r="C86" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="D86" s="13">
-        <v>44</v>
-      </c>
-      <c r="E86" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="F86" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="G86" s="14" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="87" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B86" s="44"/>
+      <c r="C86" s="44"/>
+      <c r="D86" s="44"/>
+      <c r="E86" s="44"/>
+      <c r="F86" s="44"/>
+      <c r="G86" s="44"/>
+    </row>
+    <row r="87" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="52"/>
-      <c r="B87" s="44"/>
-      <c r="C87" s="44"/>
-      <c r="D87" s="44"/>
-      <c r="E87" s="44"/>
-      <c r="F87" s="44"/>
-      <c r="G87" s="44"/>
+      <c r="B87" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="C87" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="D87" s="21">
+        <v>36</v>
+      </c>
+      <c r="E87" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="F87" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="G87" s="18" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="88" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="52"/>
-      <c r="B88" s="22" t="s">
-        <v>14</v>
-      </c>
+      <c r="B88" s="34"/>
       <c r="C88" s="9" t="s">
-        <v>59</v>
+        <v>156</v>
       </c>
       <c r="D88" s="21">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E88" s="11" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="F88" s="11" t="s">
         <v>79</v>
       </c>
       <c r="G88" s="18" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="89" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A89" s="52"/>
-      <c r="B89" s="34"/>
-      <c r="C89" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="D89" s="21">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="44"/>
+      <c r="B89" s="44"/>
+      <c r="C89" s="44"/>
+      <c r="D89" s="44"/>
+      <c r="E89" s="44"/>
+      <c r="F89" s="44"/>
+      <c r="G89" s="44"/>
+    </row>
+    <row r="90" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A90" s="53" t="s">
+        <v>25</v>
+      </c>
+      <c r="B90" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C90" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="D90" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="E90" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="F90" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="G90" s="9" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A91" s="53"/>
+      <c r="B91" s="12"/>
+      <c r="C91" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="D91" s="23">
         <v>20</v>
       </c>
-      <c r="E89" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="F89" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="G89" s="18" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="44"/>
-      <c r="B90" s="44"/>
-      <c r="C90" s="44"/>
-      <c r="D90" s="44"/>
-      <c r="E90" s="44"/>
-      <c r="F90" s="44"/>
-      <c r="G90" s="44"/>
-    </row>
-    <row r="91" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A91" s="53" t="s">
-        <v>25</v>
-      </c>
-      <c r="B91" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="C91" s="18" t="s">
-        <v>60</v>
-      </c>
-      <c r="D91" s="17" t="s">
-        <v>89</v>
-      </c>
       <c r="E91" s="11" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F91" s="18" t="s">
         <v>88</v>
       </c>
       <c r="G91" s="9" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
     </row>
     <row r="92" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="53"/>
-      <c r="B92" s="12"/>
-      <c r="C92" s="9" t="s">
-        <v>160</v>
+      <c r="B92" s="35"/>
+      <c r="C92" s="18" t="s">
+        <v>159</v>
       </c>
       <c r="D92" s="23">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E92" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="F92" s="18" t="s">
-        <v>88</v>
-      </c>
-      <c r="G92" s="9" t="s">
-        <v>98</v>
+        <v>50</v>
+      </c>
+      <c r="F92" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="G92" s="14" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="93" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="53"/>
       <c r="B93" s="35"/>
-      <c r="C93" s="18" t="s">
-        <v>162</v>
+      <c r="C93" s="9" t="s">
+        <v>158</v>
       </c>
       <c r="D93" s="23">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="E93" s="11" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="F93" s="14" t="s">
         <v>90</v>
       </c>
       <c r="G93" s="14" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="53"/>
+      <c r="B94" s="44"/>
+      <c r="C94" s="44"/>
+      <c r="D94" s="44"/>
+      <c r="E94" s="44"/>
+      <c r="F94" s="44"/>
+      <c r="G94" s="44"/>
+    </row>
+    <row r="95" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A95" s="53"/>
+      <c r="B95" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C95" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="D95" s="23">
+        <v>12</v>
+      </c>
+      <c r="E95" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="F95" s="14" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="94" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A94" s="53"/>
-      <c r="B94" s="35"/>
-      <c r="C94" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="D94" s="23">
-        <v>48</v>
-      </c>
-      <c r="E94" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="F94" s="14" t="s">
+      <c r="G95" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="G94" s="14" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="95" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A95" s="53"/>
-      <c r="B95" s="44"/>
-      <c r="C95" s="44"/>
-      <c r="D95" s="44"/>
-      <c r="E95" s="44"/>
-      <c r="F95" s="44"/>
-      <c r="G95" s="44"/>
     </row>
     <row r="96" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="53"/>
-      <c r="B96" s="12" t="s">
-        <v>11</v>
-      </c>
+      <c r="B96" s="35"/>
       <c r="C96" s="11" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D96" s="23">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E96" s="11" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="F96" s="14" t="s">
         <v>90</v>
       </c>
       <c r="G96" s="9" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A97" s="53"/>
-      <c r="B97" s="35"/>
-      <c r="C97" s="11" t="s">
-        <v>164</v>
-      </c>
-      <c r="D97" s="23">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A97" s="44"/>
+      <c r="B97" s="44"/>
+      <c r="C97" s="44"/>
+      <c r="D97" s="44"/>
+      <c r="E97" s="44"/>
+      <c r="F97" s="44"/>
+      <c r="G97" s="44"/>
+    </row>
+    <row r="98" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A98" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="B98" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C98" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="D98" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="E98" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="F98" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="G98" s="9" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A99" s="52"/>
+      <c r="B99" s="35"/>
+      <c r="C99" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="D99" s="17">
+        <v>15</v>
+      </c>
+      <c r="E99" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="E97" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="F97" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="G97" s="9" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="98" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A98" s="44"/>
-      <c r="B98" s="44"/>
-      <c r="C98" s="44"/>
-      <c r="D98" s="44"/>
-      <c r="E98" s="44"/>
-      <c r="F98" s="44"/>
-      <c r="G98" s="44"/>
-    </row>
-    <row r="99" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A99" s="52" t="s">
-        <v>26</v>
-      </c>
-      <c r="B99" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C99" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="D99" s="17" t="s">
-        <v>99</v>
-      </c>
-      <c r="E99" s="11" t="s">
-        <v>29</v>
-      </c>
       <c r="F99" s="18" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G99" s="9" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="100" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100" s="52"/>
       <c r="B100" s="35"/>
-      <c r="C100" s="9" t="s">
-        <v>165</v>
-      </c>
-      <c r="D100" s="17">
+      <c r="C100" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="D100" s="23">
+        <v>48</v>
+      </c>
+      <c r="E100" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="F100" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="G100" s="9" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A101" s="52"/>
+      <c r="B101" s="44"/>
+      <c r="C101" s="44"/>
+      <c r="D101" s="44"/>
+      <c r="E101" s="44"/>
+      <c r="F101" s="44"/>
+      <c r="G101" s="44"/>
+    </row>
+    <row r="102" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A102" s="52"/>
+      <c r="B102" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E100" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="F100" s="18" t="s">
-        <v>100</v>
-      </c>
-      <c r="G100" s="9" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="101" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A101" s="52"/>
-      <c r="B101" s="35"/>
-      <c r="C101" s="11" t="s">
-        <v>166</v>
-      </c>
-      <c r="D101" s="23">
-        <v>48</v>
-      </c>
-      <c r="E101" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="F101" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="G101" s="9" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="102" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A102" s="52"/>
-      <c r="B102" s="44"/>
-      <c r="C102" s="44"/>
-      <c r="D102" s="44"/>
-      <c r="E102" s="44"/>
-      <c r="F102" s="44"/>
-      <c r="G102" s="44"/>
+      <c r="C102" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="D102" s="23">
+        <v>40</v>
+      </c>
+      <c r="E102" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="F102" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="G102" s="9" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="103" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103" s="52"/>
-      <c r="B103" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C103" s="9" t="s">
-        <v>167</v>
+      <c r="B103" s="12"/>
+      <c r="C103" s="11" t="s">
+        <v>64</v>
       </c>
       <c r="D103" s="23">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="E103" s="11" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F103" s="14" t="s">
         <v>101</v>
       </c>
       <c r="G103" s="9" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="104" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A104" s="52"/>
       <c r="B104" s="12"/>
-      <c r="C104" s="11" t="s">
-        <v>64</v>
+      <c r="C104" s="9" t="s">
+        <v>165</v>
       </c>
       <c r="D104" s="23">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E104" s="11" t="s">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="F104" s="14" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G104" s="9" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="105" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A105" s="52"/>
       <c r="B105" s="12"/>
-      <c r="C105" s="9" t="s">
-        <v>168</v>
+      <c r="C105" s="11" t="s">
+        <v>166</v>
       </c>
       <c r="D105" s="23">
-        <v>15</v>
+        <v>65</v>
       </c>
       <c r="E105" s="11" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F105" s="14" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G105" s="9" t="s">
-        <v>100</v>
+        <v>118</v>
       </c>
     </row>
     <row r="106" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A106" s="52"/>
       <c r="B106" s="12"/>
-      <c r="C106" s="11" t="s">
-        <v>169</v>
+      <c r="C106" s="9" t="s">
+        <v>167</v>
       </c>
       <c r="D106" s="23">
-        <v>65</v>
+        <v>22</v>
       </c>
       <c r="E106" s="11" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="F106" s="14" t="s">
-        <v>102</v>
+        <v>88</v>
       </c>
       <c r="G106" s="9" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
     </row>
     <row r="107" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A107" s="52"/>
-      <c r="B107" s="12"/>
-      <c r="C107" s="9" t="s">
-        <v>170</v>
-      </c>
-      <c r="D107" s="23">
-        <v>22</v>
+      <c r="B107" s="35"/>
+      <c r="C107" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="D107" s="23" t="s">
+        <v>103</v>
       </c>
       <c r="E107" s="11" t="s">
-        <v>66</v>
+        <v>32</v>
       </c>
       <c r="F107" s="14" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="G107" s="9" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="108" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="52"/>
-      <c r="B108" s="35"/>
-      <c r="C108" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="D108" s="23" t="s">
-        <v>103</v>
-      </c>
-      <c r="E108" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="F108" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="G108" s="9" t="s">
-        <v>73</v>
-      </c>
+      <c r="B108" s="44"/>
+      <c r="C108" s="44"/>
+      <c r="D108" s="44"/>
+      <c r="E108" s="44"/>
+      <c r="F108" s="44"/>
+      <c r="G108" s="44"/>
     </row>
     <row r="109" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="52"/>
-      <c r="B109" s="44"/>
-      <c r="C109" s="44"/>
-      <c r="D109" s="44"/>
-      <c r="E109" s="44"/>
-      <c r="F109" s="44"/>
-      <c r="G109" s="44"/>
+      <c r="B109" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="C109" s="51" t="s">
+        <v>9</v>
+      </c>
+      <c r="D109" s="51"/>
+      <c r="E109" s="51"/>
+      <c r="F109" s="51"/>
+      <c r="G109" s="51"/>
     </row>
     <row r="110" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A110" s="52"/>
-      <c r="B110" s="22" t="s">
+      <c r="A110" s="33"/>
+      <c r="B110" s="33"/>
+      <c r="C110" s="44"/>
+      <c r="D110" s="44"/>
+      <c r="E110" s="44"/>
+      <c r="F110" s="44"/>
+      <c r="G110" s="44"/>
+    </row>
+    <row r="111" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A111" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="B111" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="C111" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="D111" s="13">
         <v>14</v>
       </c>
-      <c r="C110" s="51" t="s">
-        <v>9</v>
-      </c>
-      <c r="D110" s="51"/>
-      <c r="E110" s="51"/>
-      <c r="F110" s="51"/>
-      <c r="G110" s="51"/>
-    </row>
-    <row r="111" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A111" s="33"/>
-      <c r="B111" s="33"/>
-      <c r="C111" s="44"/>
-      <c r="D111" s="44"/>
-      <c r="E111" s="44"/>
-      <c r="F111" s="44"/>
-      <c r="G111" s="44"/>
+      <c r="E111" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="F111" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="G111" s="9" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="112" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A112" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="B112" s="35" t="s">
-        <v>19</v>
-      </c>
+      <c r="A112" s="52"/>
+      <c r="B112" s="35"/>
       <c r="C112" s="9" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D112" s="13">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E112" s="11" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F112" s="14" t="s">
         <v>104</v>
       </c>
       <c r="G112" s="9" t="s">
-        <v>73</v>
+        <v>104</v>
       </c>
     </row>
     <row r="113" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A113" s="52"/>
       <c r="B113" s="35"/>
-      <c r="C113" s="9" t="s">
-        <v>172</v>
+      <c r="C113" s="11" t="s">
+        <v>170</v>
       </c>
       <c r="D113" s="13">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="E113" s="11" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F113" s="14" t="s">
-        <v>104</v>
+        <v>83</v>
       </c>
       <c r="G113" s="9" t="s">
-        <v>104</v>
+        <v>83</v>
       </c>
     </row>
     <row r="114" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A114" s="52"/>
       <c r="B114" s="35"/>
       <c r="C114" s="11" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D114" s="13">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E114" s="11" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="F114" s="14" t="s">
-        <v>83</v>
+        <v>106</v>
       </c>
       <c r="G114" s="9" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="115" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A115" s="52"/>
-      <c r="B115" s="35"/>
-      <c r="C115" s="11" t="s">
-        <v>174</v>
-      </c>
-      <c r="D115" s="13">
-        <v>22</v>
-      </c>
-      <c r="E115" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="F115" s="14" t="s">
+      <c r="B115" s="33"/>
+      <c r="C115" s="44"/>
+      <c r="D115" s="44"/>
+      <c r="E115" s="44"/>
+      <c r="F115" s="44"/>
+      <c r="G115" s="44"/>
+    </row>
+    <row r="116" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A116" s="52"/>
+      <c r="B116" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="C116" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="D116" s="13">
+        <v>16</v>
+      </c>
+      <c r="E116" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F116" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="G116" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="G115" s="9" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="116" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A116" s="52"/>
-      <c r="B116" s="33"/>
-      <c r="C116" s="44"/>
-      <c r="D116" s="44"/>
-      <c r="E116" s="44"/>
-      <c r="F116" s="44"/>
-      <c r="G116" s="44"/>
     </row>
     <row r="117" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A117" s="52"/>
-      <c r="B117" s="22" t="s">
-        <v>10</v>
-      </c>
+      <c r="B117" s="35"/>
       <c r="C117" s="9" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D117" s="13">
-        <v>16</v>
-      </c>
-      <c r="E117" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="E117" s="11" t="s">
+        <v>35</v>
       </c>
       <c r="F117" s="14" t="s">
         <v>104</v>
       </c>
       <c r="G117" s="9" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="118" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A118" s="52"/>
       <c r="B118" s="35"/>
       <c r="C118" s="9" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D118" s="13">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="E118" s="11" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F118" s="14" t="s">
         <v>104</v>
       </c>
       <c r="G118" s="9" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="119" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="52"/>
-      <c r="B119" s="35"/>
-      <c r="C119" s="9" t="s">
-        <v>177</v>
-      </c>
-      <c r="D119" s="13">
-        <v>19</v>
-      </c>
-      <c r="E119" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="F119" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="G119" s="9" t="s">
-        <v>83</v>
-      </c>
+      <c r="B119" s="33"/>
+      <c r="C119" s="44"/>
+      <c r="D119" s="44"/>
+      <c r="E119" s="44"/>
+      <c r="F119" s="44"/>
+      <c r="G119" s="44"/>
     </row>
     <row r="120" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="52"/>
-      <c r="B120" s="33"/>
-      <c r="C120" s="44"/>
-      <c r="D120" s="44"/>
-      <c r="E120" s="44"/>
-      <c r="F120" s="44"/>
-      <c r="G120" s="44"/>
+      <c r="B120" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C120" s="51" t="s">
+        <v>9</v>
+      </c>
+      <c r="D120" s="51"/>
+      <c r="E120" s="51"/>
+      <c r="F120" s="51"/>
+      <c r="G120" s="51"/>
     </row>
     <row r="121" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A121" s="52"/>
-      <c r="B121" s="22" t="s">
-        <v>11</v>
-      </c>
-      <c r="C121" s="51" t="s">
-        <v>9</v>
-      </c>
-      <c r="D121" s="51"/>
-      <c r="E121" s="51"/>
-      <c r="F121" s="51"/>
-      <c r="G121" s="51"/>
-    </row>
-    <row r="122" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B121" s="33"/>
+      <c r="C121" s="44"/>
+      <c r="D121" s="44"/>
+      <c r="E121" s="44"/>
+      <c r="F121" s="44"/>
+      <c r="G121" s="44"/>
+    </row>
+    <row r="122" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A122" s="52"/>
-      <c r="B122" s="33"/>
-      <c r="C122" s="44"/>
-      <c r="D122" s="44"/>
-      <c r="E122" s="44"/>
-      <c r="F122" s="44"/>
-      <c r="G122" s="44"/>
-    </row>
-    <row r="123" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A123" s="52"/>
-      <c r="B123" s="12" t="s">
+      <c r="B122" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C123" s="41" t="s">
+      <c r="C122" s="41" t="s">
         <v>111</v>
       </c>
-      <c r="D123" s="13">
+      <c r="D122" s="13">
         <v>41</v>
       </c>
-      <c r="E123" s="9" t="s">
+      <c r="E122" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="F123" s="14" t="s">
+      <c r="F122" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="G123" s="14" t="s">
+      <c r="G122" s="14" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="124" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A124" s="36"/>
-      <c r="B124" s="36"/>
-      <c r="C124" s="37"/>
-      <c r="D124" s="37"/>
-      <c r="E124" s="37"/>
-      <c r="F124" s="37"/>
-      <c r="G124" s="37"/>
+    <row r="123" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A123" s="36"/>
+      <c r="B123" s="36"/>
+      <c r="C123" s="37"/>
+      <c r="D123" s="37"/>
+      <c r="E123" s="37"/>
+      <c r="F123" s="37"/>
+      <c r="G123" s="37"/>
+    </row>
+    <row r="124" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A124" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="B124" s="35" t="s">
+        <v>177</v>
+      </c>
+      <c r="C124" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="D124" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="E124" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="F124" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="G124" s="9" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="125" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A125" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="B125" s="35" t="s">
-        <v>180</v>
-      </c>
+      <c r="A125" s="52"/>
+      <c r="B125" s="35"/>
       <c r="C125" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="D125" s="13" t="s">
-        <v>108</v>
+        <v>175</v>
+      </c>
+      <c r="D125" s="13">
+        <v>15</v>
       </c>
       <c r="E125" s="11" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F125" s="14" t="s">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="G125" s="9" t="s">
-        <v>109</v>
+        <v>90</v>
       </c>
     </row>
     <row r="126" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A126" s="52"/>
       <c r="B126" s="35"/>
       <c r="C126" s="9" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="D126" s="13">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="E126" s="11" t="s">
-        <v>34</v>
+        <v>51</v>
       </c>
       <c r="F126" s="14" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="G126" s="9" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
     </row>
     <row r="127" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A127" s="52"/>
       <c r="B127" s="35"/>
       <c r="C127" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="D127" s="13">
-        <v>59</v>
+        <v>68</v>
+      </c>
+      <c r="D127" s="13" t="s">
+        <v>107</v>
       </c>
       <c r="E127" s="11" t="s">
-        <v>51</v>
+        <v>31</v>
       </c>
       <c r="F127" s="14" t="s">
-        <v>74</v>
+        <v>101</v>
       </c>
       <c r="G127" s="9" t="s">
-        <v>74</v>
+        <v>101</v>
       </c>
     </row>
     <row r="128" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A128" s="52"/>
       <c r="B128" s="35"/>
       <c r="C128" s="9" t="s">
-        <v>68</v>
+        <v>184</v>
       </c>
       <c r="D128" s="13" t="s">
-        <v>107</v>
+        <v>185</v>
       </c>
       <c r="E128" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F128" s="14" t="s">
-        <v>101</v>
+        <v>186</v>
       </c>
       <c r="G128" s="9" t="s">
-        <v>101</v>
+        <v>119</v>
       </c>
     </row>
     <row r="129" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A129" s="52"/>
       <c r="B129" s="35"/>
       <c r="C129" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="D129" s="13" t="s">
-        <v>188</v>
+        <v>120</v>
+      </c>
+      <c r="D129" s="13">
+        <v>34</v>
       </c>
       <c r="E129" s="11" t="s">
-        <v>32</v>
+        <v>121</v>
       </c>
       <c r="F129" s="14" t="s">
-        <v>189</v>
+        <v>75</v>
       </c>
       <c r="G129" s="9" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="130" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7" ht="15.5" x14ac:dyDescent="0.3">
       <c r="A130" s="52"/>
-      <c r="B130" s="35"/>
-      <c r="C130" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="D130" s="13">
-        <v>34</v>
-      </c>
-      <c r="E130" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="F130" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="G130" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="131" spans="1:7" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A131" s="52"/>
-      <c r="B131" s="33"/>
-      <c r="C131" s="44"/>
-      <c r="D131" s="44"/>
-      <c r="E131" s="44"/>
-      <c r="F131" s="44"/>
-      <c r="G131" s="44"/>
+      <c r="B130" s="33"/>
+      <c r="C130" s="44"/>
+      <c r="D130" s="44"/>
+      <c r="E130" s="44"/>
+      <c r="F130" s="44"/>
+      <c r="G130" s="44"/>
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="B109:G109"/>
+    <mergeCell ref="B108:G108"/>
     <mergeCell ref="B15:G15"/>
     <mergeCell ref="A20:G20"/>
     <mergeCell ref="B11:G11"/>
     <mergeCell ref="B52:G52"/>
-    <mergeCell ref="B80:G80"/>
+    <mergeCell ref="B79:G79"/>
     <mergeCell ref="B57:G57"/>
     <mergeCell ref="A54:G54"/>
     <mergeCell ref="B22:B25"/>
@@ -3512,40 +3487,40 @@
     <mergeCell ref="C21:F21"/>
     <mergeCell ref="B26:G26"/>
     <mergeCell ref="A32:A40"/>
-    <mergeCell ref="A81:A89"/>
-    <mergeCell ref="A91:A97"/>
-    <mergeCell ref="A125:A131"/>
-    <mergeCell ref="C131:G131"/>
-    <mergeCell ref="A112:A123"/>
+    <mergeCell ref="A80:A88"/>
+    <mergeCell ref="A90:A96"/>
+    <mergeCell ref="A124:A130"/>
+    <mergeCell ref="C130:G130"/>
+    <mergeCell ref="A111:A122"/>
     <mergeCell ref="A9:A18"/>
     <mergeCell ref="A21:A30"/>
     <mergeCell ref="A42:A53"/>
-    <mergeCell ref="A55:A79"/>
-    <mergeCell ref="A98:G98"/>
+    <mergeCell ref="A55:A78"/>
+    <mergeCell ref="A97:G97"/>
     <mergeCell ref="B50:G50"/>
     <mergeCell ref="B46:G46"/>
     <mergeCell ref="A41:G41"/>
     <mergeCell ref="B38:G38"/>
     <mergeCell ref="B36:G36"/>
     <mergeCell ref="A31:G31"/>
-    <mergeCell ref="C120:G120"/>
-    <mergeCell ref="B95:G95"/>
-    <mergeCell ref="C111:G111"/>
+    <mergeCell ref="C119:G119"/>
+    <mergeCell ref="B94:G94"/>
+    <mergeCell ref="C110:G110"/>
     <mergeCell ref="C9:F9"/>
     <mergeCell ref="C37:F37"/>
-    <mergeCell ref="C122:G122"/>
-    <mergeCell ref="C110:G110"/>
     <mergeCell ref="C121:G121"/>
+    <mergeCell ref="C109:G109"/>
+    <mergeCell ref="C120:G120"/>
     <mergeCell ref="C51:G51"/>
     <mergeCell ref="C53:G53"/>
-    <mergeCell ref="B102:G102"/>
-    <mergeCell ref="C116:G116"/>
-    <mergeCell ref="B72:G72"/>
-    <mergeCell ref="A90:G90"/>
-    <mergeCell ref="B87:G87"/>
-    <mergeCell ref="B84:G84"/>
-    <mergeCell ref="B77:F77"/>
-    <mergeCell ref="A99:A110"/>
+    <mergeCell ref="B101:G101"/>
+    <mergeCell ref="C115:G115"/>
+    <mergeCell ref="B71:G71"/>
+    <mergeCell ref="A89:G89"/>
+    <mergeCell ref="B86:G86"/>
+    <mergeCell ref="B83:G83"/>
+    <mergeCell ref="B76:F76"/>
+    <mergeCell ref="A98:A109"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.625" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="53" fitToHeight="0" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Update data in master_schedule.xlsx to reflect the latest schedule changes.
</commit_message>
<xml_diff>
--- a/storage/app/master_schedule.xlsx
+++ b/storage/app/master_schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Laravel Projects\lecturer-invigilation-portal\storage\app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F767CEB5-7019-43BE-917A-548DA4677275}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{001E1E87-4A8F-4098-BE1A-E81A27273751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -895,6 +895,15 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -904,6 +913,15 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -915,24 +933,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1437,12 +1437,12 @@
       <c r="B9" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="45" t="s">
+      <c r="C9" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="46"/>
-      <c r="E9" s="46"/>
-      <c r="F9" s="47"/>
+      <c r="D9" s="49"/>
+      <c r="E9" s="49"/>
+      <c r="F9" s="50"/>
       <c r="G9" s="18"/>
     </row>
     <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1625,17 +1625,17 @@
       <c r="B21" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="45" t="s">
+      <c r="C21" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="D21" s="46"/>
-      <c r="E21" s="46"/>
-      <c r="F21" s="47"/>
+      <c r="D21" s="49"/>
+      <c r="E21" s="49"/>
+      <c r="F21" s="50"/>
       <c r="G21" s="18"/>
     </row>
     <row r="22" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="53"/>
-      <c r="B22" s="55" t="s">
+      <c r="B22" s="46" t="s">
         <v>36</v>
       </c>
       <c r="C22" s="39" t="s">
@@ -1656,7 +1656,7 @@
     </row>
     <row r="23" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="53"/>
-      <c r="B23" s="55"/>
+      <c r="B23" s="46"/>
       <c r="C23" s="39" t="s">
         <v>81</v>
       </c>
@@ -1675,7 +1675,7 @@
     </row>
     <row r="24" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="53"/>
-      <c r="B24" s="55"/>
+      <c r="B24" s="46"/>
       <c r="C24" s="39" t="s">
         <v>82</v>
       </c>
@@ -1694,7 +1694,7 @@
     </row>
     <row r="25" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="53"/>
-      <c r="B25" s="55"/>
+      <c r="B25" s="46"/>
       <c r="C25" s="39" t="s">
         <v>130</v>
       </c>
@@ -1722,7 +1722,7 @@
     </row>
     <row r="27" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="53"/>
-      <c r="B27" s="56" t="s">
+      <c r="B27" s="47" t="s">
         <v>11</v>
       </c>
       <c r="C27" s="9" t="s">
@@ -1743,7 +1743,7 @@
     </row>
     <row r="28" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="53"/>
-      <c r="B28" s="56"/>
+      <c r="B28" s="47"/>
       <c r="C28" s="9" t="s">
         <v>133</v>
       </c>
@@ -1762,7 +1762,7 @@
     </row>
     <row r="29" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="53"/>
-      <c r="B29" s="56"/>
+      <c r="B29" s="47"/>
       <c r="C29" s="9" t="s">
         <v>40</v>
       </c>
@@ -1781,7 +1781,7 @@
     </row>
     <row r="30" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="53"/>
-      <c r="B30" s="56"/>
+      <c r="B30" s="47"/>
       <c r="C30" s="9" t="s">
         <v>41</v>
       </c>
@@ -1799,16 +1799,16 @@
       </c>
     </row>
     <row r="31" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="54"/>
-      <c r="B31" s="54"/>
-      <c r="C31" s="54"/>
-      <c r="D31" s="54"/>
-      <c r="E31" s="54"/>
-      <c r="F31" s="54"/>
-      <c r="G31" s="54"/>
+      <c r="A31" s="45"/>
+      <c r="B31" s="45"/>
+      <c r="C31" s="45"/>
+      <c r="D31" s="45"/>
+      <c r="E31" s="45"/>
+      <c r="F31" s="45"/>
+      <c r="G31" s="45"/>
     </row>
     <row r="32" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="57" t="s">
+      <c r="A32" s="51" t="s">
         <v>22</v>
       </c>
       <c r="B32" s="22" t="s">
@@ -1831,7 +1831,7 @@
       </c>
     </row>
     <row r="33" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="57"/>
+      <c r="A33" s="51"/>
       <c r="B33" s="22"/>
       <c r="C33" s="9" t="s">
         <v>92</v>
@@ -1850,7 +1850,7 @@
       </c>
     </row>
     <row r="34" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="57"/>
+      <c r="A34" s="51"/>
       <c r="B34" s="22"/>
       <c r="C34" s="9" t="s">
         <v>93</v>
@@ -1869,7 +1869,7 @@
       </c>
     </row>
     <row r="35" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="57"/>
+      <c r="A35" s="51"/>
       <c r="B35" s="22"/>
       <c r="C35" s="9" t="s">
         <v>134</v>
@@ -1888,7 +1888,7 @@
       </c>
     </row>
     <row r="36" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="57"/>
+      <c r="A36" s="51"/>
       <c r="B36" s="44"/>
       <c r="C36" s="44"/>
       <c r="D36" s="44"/>
@@ -1897,20 +1897,20 @@
       <c r="G36" s="44"/>
     </row>
     <row r="37" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="57"/>
+      <c r="A37" s="51"/>
       <c r="B37" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C37" s="48" t="s">
+      <c r="C37" s="54" t="s">
         <v>9</v>
       </c>
-      <c r="D37" s="49"/>
-      <c r="E37" s="49"/>
-      <c r="F37" s="50"/>
+      <c r="D37" s="55"/>
+      <c r="E37" s="55"/>
+      <c r="F37" s="56"/>
       <c r="G37" s="40"/>
     </row>
     <row r="38" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="57"/>
+      <c r="A38" s="51"/>
       <c r="B38" s="44"/>
       <c r="C38" s="44"/>
       <c r="D38" s="44"/>
@@ -1919,7 +1919,7 @@
       <c r="G38" s="44"/>
     </row>
     <row r="39" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="57"/>
+      <c r="A39" s="51"/>
       <c r="B39" s="22" t="s">
         <v>14</v>
       </c>
@@ -1940,7 +1940,7 @@
       </c>
     </row>
     <row r="40" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="57"/>
+      <c r="A40" s="51"/>
       <c r="B40" s="25"/>
       <c r="C40" s="9" t="s">
         <v>135</v>
@@ -2129,13 +2129,13 @@
       <c r="B51" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="C51" s="51" t="s">
+      <c r="C51" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="D51" s="51"/>
-      <c r="E51" s="51"/>
-      <c r="F51" s="51"/>
-      <c r="G51" s="51"/>
+      <c r="D51" s="57"/>
+      <c r="E51" s="57"/>
+      <c r="F51" s="57"/>
+      <c r="G51" s="57"/>
     </row>
     <row r="52" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="52"/>
@@ -2151,22 +2151,22 @@
       <c r="B53" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="C53" s="51" t="s">
+      <c r="C53" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="D53" s="51"/>
-      <c r="E53" s="51"/>
-      <c r="F53" s="51"/>
-      <c r="G53" s="51"/>
+      <c r="D53" s="57"/>
+      <c r="E53" s="57"/>
+      <c r="F53" s="57"/>
+      <c r="G53" s="57"/>
     </row>
     <row r="54" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="54"/>
-      <c r="B54" s="54"/>
-      <c r="C54" s="54"/>
-      <c r="D54" s="54"/>
-      <c r="E54" s="54"/>
-      <c r="F54" s="54"/>
-      <c r="G54" s="54"/>
+      <c r="A54" s="45"/>
+      <c r="B54" s="45"/>
+      <c r="C54" s="45"/>
+      <c r="D54" s="45"/>
+      <c r="E54" s="45"/>
+      <c r="F54" s="45"/>
+      <c r="G54" s="45"/>
     </row>
     <row r="55" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="52" t="s">
@@ -3119,13 +3119,13 @@
       <c r="B109" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C109" s="51" t="s">
+      <c r="C109" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="D109" s="51"/>
-      <c r="E109" s="51"/>
-      <c r="F109" s="51"/>
-      <c r="G109" s="51"/>
+      <c r="D109" s="57"/>
+      <c r="E109" s="57"/>
+      <c r="F109" s="57"/>
+      <c r="G109" s="57"/>
     </row>
     <row r="110" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="33"/>
@@ -3298,13 +3298,13 @@
       <c r="B120" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="C120" s="51" t="s">
+      <c r="C120" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="D120" s="51"/>
-      <c r="E120" s="51"/>
-      <c r="F120" s="51"/>
-      <c r="G120" s="51"/>
+      <c r="D120" s="57"/>
+      <c r="E120" s="57"/>
+      <c r="F120" s="57"/>
+      <c r="G120" s="57"/>
     </row>
     <row r="121" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A121" s="52"/>
@@ -3474,21 +3474,22 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="B108:G108"/>
-    <mergeCell ref="B15:G15"/>
-    <mergeCell ref="A20:G20"/>
-    <mergeCell ref="B11:G11"/>
-    <mergeCell ref="B52:G52"/>
-    <mergeCell ref="B79:G79"/>
-    <mergeCell ref="B57:G57"/>
-    <mergeCell ref="A54:G54"/>
-    <mergeCell ref="B22:B25"/>
-    <mergeCell ref="B27:B30"/>
-    <mergeCell ref="C21:F21"/>
-    <mergeCell ref="B26:G26"/>
-    <mergeCell ref="A32:A40"/>
-    <mergeCell ref="A80:A88"/>
-    <mergeCell ref="A90:A96"/>
+    <mergeCell ref="C110:G110"/>
+    <mergeCell ref="C9:F9"/>
+    <mergeCell ref="C37:F37"/>
+    <mergeCell ref="C121:G121"/>
+    <mergeCell ref="C109:G109"/>
+    <mergeCell ref="C120:G120"/>
+    <mergeCell ref="C51:G51"/>
+    <mergeCell ref="C53:G53"/>
+    <mergeCell ref="B101:G101"/>
+    <mergeCell ref="C115:G115"/>
+    <mergeCell ref="B71:G71"/>
+    <mergeCell ref="A89:G89"/>
+    <mergeCell ref="B86:G86"/>
+    <mergeCell ref="B83:G83"/>
+    <mergeCell ref="B76:F76"/>
+    <mergeCell ref="A98:A109"/>
     <mergeCell ref="A124:A130"/>
     <mergeCell ref="C130:G130"/>
     <mergeCell ref="A111:A122"/>
@@ -3505,22 +3506,21 @@
     <mergeCell ref="A31:G31"/>
     <mergeCell ref="C119:G119"/>
     <mergeCell ref="B94:G94"/>
-    <mergeCell ref="C110:G110"/>
-    <mergeCell ref="C9:F9"/>
-    <mergeCell ref="C37:F37"/>
-    <mergeCell ref="C121:G121"/>
-    <mergeCell ref="C109:G109"/>
-    <mergeCell ref="C120:G120"/>
-    <mergeCell ref="C51:G51"/>
-    <mergeCell ref="C53:G53"/>
-    <mergeCell ref="B101:G101"/>
-    <mergeCell ref="C115:G115"/>
-    <mergeCell ref="B71:G71"/>
-    <mergeCell ref="A89:G89"/>
-    <mergeCell ref="B86:G86"/>
-    <mergeCell ref="B83:G83"/>
-    <mergeCell ref="B76:F76"/>
-    <mergeCell ref="A98:A109"/>
+    <mergeCell ref="B108:G108"/>
+    <mergeCell ref="B15:G15"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="B11:G11"/>
+    <mergeCell ref="B52:G52"/>
+    <mergeCell ref="B79:G79"/>
+    <mergeCell ref="B57:G57"/>
+    <mergeCell ref="A54:G54"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="B27:B30"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="B26:G26"/>
+    <mergeCell ref="A32:A40"/>
+    <mergeCell ref="A80:A88"/>
+    <mergeCell ref="A90:A96"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.625" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="53" fitToHeight="0" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Update excel data on Alex Wambua
</commit_message>
<xml_diff>
--- a/storage/app/master_schedule.xlsx
+++ b/storage/app/master_schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Laravel Projects\lecturer-invigilation-portal\storage\app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{001E1E87-4A8F-4098-BE1A-E81A27273751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9BA1745-4CE0-40B5-9921-1FE7F524238E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -895,6 +895,33 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -904,35 +931,8 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1437,12 +1437,12 @@
       <c r="B9" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="48" t="s">
+      <c r="C9" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="49"/>
-      <c r="E9" s="49"/>
-      <c r="F9" s="50"/>
+      <c r="D9" s="46"/>
+      <c r="E9" s="46"/>
+      <c r="F9" s="47"/>
       <c r="G9" s="18"/>
     </row>
     <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1625,17 +1625,17 @@
       <c r="B21" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="48" t="s">
+      <c r="C21" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="D21" s="49"/>
-      <c r="E21" s="49"/>
-      <c r="F21" s="50"/>
+      <c r="D21" s="46"/>
+      <c r="E21" s="46"/>
+      <c r="F21" s="47"/>
       <c r="G21" s="18"/>
     </row>
     <row r="22" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="53"/>
-      <c r="B22" s="46" t="s">
+      <c r="B22" s="55" t="s">
         <v>36</v>
       </c>
       <c r="C22" s="39" t="s">
@@ -1656,7 +1656,7 @@
     </row>
     <row r="23" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="53"/>
-      <c r="B23" s="46"/>
+      <c r="B23" s="55"/>
       <c r="C23" s="39" t="s">
         <v>81</v>
       </c>
@@ -1675,7 +1675,7 @@
     </row>
     <row r="24" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="53"/>
-      <c r="B24" s="46"/>
+      <c r="B24" s="55"/>
       <c r="C24" s="39" t="s">
         <v>82</v>
       </c>
@@ -1694,7 +1694,7 @@
     </row>
     <row r="25" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="53"/>
-      <c r="B25" s="46"/>
+      <c r="B25" s="55"/>
       <c r="C25" s="39" t="s">
         <v>130</v>
       </c>
@@ -1722,7 +1722,7 @@
     </row>
     <row r="27" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="53"/>
-      <c r="B27" s="47" t="s">
+      <c r="B27" s="56" t="s">
         <v>11</v>
       </c>
       <c r="C27" s="9" t="s">
@@ -1743,7 +1743,7 @@
     </row>
     <row r="28" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="53"/>
-      <c r="B28" s="47"/>
+      <c r="B28" s="56"/>
       <c r="C28" s="9" t="s">
         <v>133</v>
       </c>
@@ -1762,7 +1762,7 @@
     </row>
     <row r="29" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="53"/>
-      <c r="B29" s="47"/>
+      <c r="B29" s="56"/>
       <c r="C29" s="9" t="s">
         <v>40</v>
       </c>
@@ -1781,7 +1781,7 @@
     </row>
     <row r="30" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="53"/>
-      <c r="B30" s="47"/>
+      <c r="B30" s="56"/>
       <c r="C30" s="9" t="s">
         <v>41</v>
       </c>
@@ -1799,16 +1799,16 @@
       </c>
     </row>
     <row r="31" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="45"/>
-      <c r="B31" s="45"/>
-      <c r="C31" s="45"/>
-      <c r="D31" s="45"/>
-      <c r="E31" s="45"/>
-      <c r="F31" s="45"/>
-      <c r="G31" s="45"/>
+      <c r="A31" s="54"/>
+      <c r="B31" s="54"/>
+      <c r="C31" s="54"/>
+      <c r="D31" s="54"/>
+      <c r="E31" s="54"/>
+      <c r="F31" s="54"/>
+      <c r="G31" s="54"/>
     </row>
     <row r="32" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="51" t="s">
+      <c r="A32" s="57" t="s">
         <v>22</v>
       </c>
       <c r="B32" s="22" t="s">
@@ -1831,7 +1831,7 @@
       </c>
     </row>
     <row r="33" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="51"/>
+      <c r="A33" s="57"/>
       <c r="B33" s="22"/>
       <c r="C33" s="9" t="s">
         <v>92</v>
@@ -1850,7 +1850,7 @@
       </c>
     </row>
     <row r="34" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="51"/>
+      <c r="A34" s="57"/>
       <c r="B34" s="22"/>
       <c r="C34" s="9" t="s">
         <v>93</v>
@@ -1869,7 +1869,7 @@
       </c>
     </row>
     <row r="35" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="51"/>
+      <c r="A35" s="57"/>
       <c r="B35" s="22"/>
       <c r="C35" s="9" t="s">
         <v>134</v>
@@ -1888,7 +1888,7 @@
       </c>
     </row>
     <row r="36" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="51"/>
+      <c r="A36" s="57"/>
       <c r="B36" s="44"/>
       <c r="C36" s="44"/>
       <c r="D36" s="44"/>
@@ -1897,20 +1897,20 @@
       <c r="G36" s="44"/>
     </row>
     <row r="37" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="51"/>
+      <c r="A37" s="57"/>
       <c r="B37" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C37" s="54" t="s">
+      <c r="C37" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="D37" s="55"/>
-      <c r="E37" s="55"/>
-      <c r="F37" s="56"/>
+      <c r="D37" s="49"/>
+      <c r="E37" s="49"/>
+      <c r="F37" s="50"/>
       <c r="G37" s="40"/>
     </row>
     <row r="38" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="51"/>
+      <c r="A38" s="57"/>
       <c r="B38" s="44"/>
       <c r="C38" s="44"/>
       <c r="D38" s="44"/>
@@ -1919,7 +1919,7 @@
       <c r="G38" s="44"/>
     </row>
     <row r="39" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="51"/>
+      <c r="A39" s="57"/>
       <c r="B39" s="22" t="s">
         <v>14</v>
       </c>
@@ -1940,7 +1940,7 @@
       </c>
     </row>
     <row r="40" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="51"/>
+      <c r="A40" s="57"/>
       <c r="B40" s="25"/>
       <c r="C40" s="9" t="s">
         <v>135</v>
@@ -2129,13 +2129,13 @@
       <c r="B51" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="C51" s="57" t="s">
+      <c r="C51" s="51" t="s">
         <v>9</v>
       </c>
-      <c r="D51" s="57"/>
-      <c r="E51" s="57"/>
-      <c r="F51" s="57"/>
-      <c r="G51" s="57"/>
+      <c r="D51" s="51"/>
+      <c r="E51" s="51"/>
+      <c r="F51" s="51"/>
+      <c r="G51" s="51"/>
     </row>
     <row r="52" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="52"/>
@@ -2151,22 +2151,22 @@
       <c r="B53" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="C53" s="57" t="s">
+      <c r="C53" s="51" t="s">
         <v>9</v>
       </c>
-      <c r="D53" s="57"/>
-      <c r="E53" s="57"/>
-      <c r="F53" s="57"/>
-      <c r="G53" s="57"/>
+      <c r="D53" s="51"/>
+      <c r="E53" s="51"/>
+      <c r="F53" s="51"/>
+      <c r="G53" s="51"/>
     </row>
     <row r="54" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="45"/>
-      <c r="B54" s="45"/>
-      <c r="C54" s="45"/>
-      <c r="D54" s="45"/>
-      <c r="E54" s="45"/>
-      <c r="F54" s="45"/>
-      <c r="G54" s="45"/>
+      <c r="A54" s="54"/>
+      <c r="B54" s="54"/>
+      <c r="C54" s="54"/>
+      <c r="D54" s="54"/>
+      <c r="E54" s="54"/>
+      <c r="F54" s="54"/>
+      <c r="G54" s="54"/>
     </row>
     <row r="55" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="52" t="s">
@@ -2446,7 +2446,7 @@
         <v>106</v>
       </c>
       <c r="G69" s="14" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
     </row>
     <row r="70" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -3119,13 +3119,13 @@
       <c r="B109" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C109" s="57" t="s">
+      <c r="C109" s="51" t="s">
         <v>9</v>
       </c>
-      <c r="D109" s="57"/>
-      <c r="E109" s="57"/>
-      <c r="F109" s="57"/>
-      <c r="G109" s="57"/>
+      <c r="D109" s="51"/>
+      <c r="E109" s="51"/>
+      <c r="F109" s="51"/>
+      <c r="G109" s="51"/>
     </row>
     <row r="110" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="33"/>
@@ -3298,13 +3298,13 @@
       <c r="B120" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="C120" s="57" t="s">
+      <c r="C120" s="51" t="s">
         <v>9</v>
       </c>
-      <c r="D120" s="57"/>
-      <c r="E120" s="57"/>
-      <c r="F120" s="57"/>
-      <c r="G120" s="57"/>
+      <c r="D120" s="51"/>
+      <c r="E120" s="51"/>
+      <c r="F120" s="51"/>
+      <c r="G120" s="51"/>
     </row>
     <row r="121" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A121" s="52"/>
@@ -3474,6 +3474,37 @@
     </row>
   </sheetData>
   <mergeCells count="47">
+    <mergeCell ref="B108:G108"/>
+    <mergeCell ref="B15:G15"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="B11:G11"/>
+    <mergeCell ref="B52:G52"/>
+    <mergeCell ref="B79:G79"/>
+    <mergeCell ref="B57:G57"/>
+    <mergeCell ref="A54:G54"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="B27:B30"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="B26:G26"/>
+    <mergeCell ref="A32:A40"/>
+    <mergeCell ref="A80:A88"/>
+    <mergeCell ref="A90:A96"/>
+    <mergeCell ref="A124:A130"/>
+    <mergeCell ref="C130:G130"/>
+    <mergeCell ref="A111:A122"/>
+    <mergeCell ref="A9:A18"/>
+    <mergeCell ref="A21:A30"/>
+    <mergeCell ref="A42:A53"/>
+    <mergeCell ref="A55:A78"/>
+    <mergeCell ref="A97:G97"/>
+    <mergeCell ref="B50:G50"/>
+    <mergeCell ref="B46:G46"/>
+    <mergeCell ref="A41:G41"/>
+    <mergeCell ref="B38:G38"/>
+    <mergeCell ref="B36:G36"/>
+    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="C119:G119"/>
+    <mergeCell ref="B94:G94"/>
     <mergeCell ref="C110:G110"/>
     <mergeCell ref="C9:F9"/>
     <mergeCell ref="C37:F37"/>
@@ -3490,37 +3521,6 @@
     <mergeCell ref="B83:G83"/>
     <mergeCell ref="B76:F76"/>
     <mergeCell ref="A98:A109"/>
-    <mergeCell ref="A124:A130"/>
-    <mergeCell ref="C130:G130"/>
-    <mergeCell ref="A111:A122"/>
-    <mergeCell ref="A9:A18"/>
-    <mergeCell ref="A21:A30"/>
-    <mergeCell ref="A42:A53"/>
-    <mergeCell ref="A55:A78"/>
-    <mergeCell ref="A97:G97"/>
-    <mergeCell ref="B50:G50"/>
-    <mergeCell ref="B46:G46"/>
-    <mergeCell ref="A41:G41"/>
-    <mergeCell ref="B38:G38"/>
-    <mergeCell ref="B36:G36"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="C119:G119"/>
-    <mergeCell ref="B94:G94"/>
-    <mergeCell ref="B108:G108"/>
-    <mergeCell ref="B15:G15"/>
-    <mergeCell ref="A20:G20"/>
-    <mergeCell ref="B11:G11"/>
-    <mergeCell ref="B52:G52"/>
-    <mergeCell ref="B79:G79"/>
-    <mergeCell ref="B57:G57"/>
-    <mergeCell ref="A54:G54"/>
-    <mergeCell ref="B22:B25"/>
-    <mergeCell ref="B27:B30"/>
-    <mergeCell ref="C21:F21"/>
-    <mergeCell ref="B26:G26"/>
-    <mergeCell ref="A32:A40"/>
-    <mergeCell ref="A80:A88"/>
-    <mergeCell ref="A90:A96"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.625" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="53" fitToHeight="0" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Update spelling in master_schedule.xlsx
</commit_message>
<xml_diff>
--- a/storage/app/master_schedule.xlsx
+++ b/storage/app/master_schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Laravel Projects\lecturer-invigilation-portal\storage\app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9BA1745-4CE0-40B5-9921-1FE7F524238E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BBE0565-CF42-444E-B64F-A43C1B94E171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="190">
   <si>
     <t>DATE</t>
   </si>
@@ -340,9 +340,6 @@
     <t>Dr. Dismus Ombuya</t>
   </si>
   <si>
-    <t>Mr. Duncan Eric Ogongi</t>
-  </si>
-  <si>
     <t>35+12+12=59</t>
   </si>
   <si>
@@ -386,9 +383,6 @@
   </si>
   <si>
     <t>32+6=38</t>
-  </si>
-  <si>
-    <t>Mr. Dancan Eric Ogonji</t>
   </si>
   <si>
     <t>Dr Watson Kanuku</t>
@@ -895,6 +889,15 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -904,6 +907,15 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -915,24 +927,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1401,7 +1395,7 @@
     <row r="7" spans="1:7" ht="17.5" x14ac:dyDescent="0.35">
       <c r="A7" s="1"/>
       <c r="B7" s="4" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C7" s="4"/>
       <c r="D7" s="7"/>
@@ -1437,12 +1431,12 @@
       <c r="B9" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="45" t="s">
+      <c r="C9" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="46"/>
-      <c r="E9" s="46"/>
-      <c r="F9" s="47"/>
+      <c r="D9" s="49"/>
+      <c r="E9" s="49"/>
+      <c r="F9" s="50"/>
       <c r="G9" s="18"/>
     </row>
     <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1469,10 +1463,10 @@
         <v>17</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>29</v>
@@ -1488,7 +1482,7 @@
       <c r="A13" s="53"/>
       <c r="B13" s="19"/>
       <c r="C13" s="9" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D13" s="13">
         <v>35</v>
@@ -1507,7 +1501,7 @@
       <c r="A14" s="53"/>
       <c r="B14" s="19"/>
       <c r="C14" s="9" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D14" s="13">
         <v>35</v>
@@ -1556,7 +1550,7 @@
       <c r="A17" s="53"/>
       <c r="B17" s="19"/>
       <c r="C17" s="11" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D17" s="21">
         <v>12</v>
@@ -1575,7 +1569,7 @@
       <c r="A18" s="53"/>
       <c r="B18" s="19"/>
       <c r="C18" s="11" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D18" s="21">
         <v>58</v>
@@ -1594,7 +1588,7 @@
       <c r="A19" s="42"/>
       <c r="B19" s="19"/>
       <c r="C19" s="11" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D19" s="21">
         <v>40</v>
@@ -1625,17 +1619,17 @@
       <c r="B21" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="45" t="s">
+      <c r="C21" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="D21" s="46"/>
-      <c r="E21" s="46"/>
-      <c r="F21" s="47"/>
+      <c r="D21" s="49"/>
+      <c r="E21" s="49"/>
+      <c r="F21" s="50"/>
       <c r="G21" s="18"/>
     </row>
     <row r="22" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="53"/>
-      <c r="B22" s="55" t="s">
+      <c r="B22" s="46" t="s">
         <v>36</v>
       </c>
       <c r="C22" s="39" t="s">
@@ -1656,7 +1650,7 @@
     </row>
     <row r="23" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="53"/>
-      <c r="B23" s="55"/>
+      <c r="B23" s="46"/>
       <c r="C23" s="39" t="s">
         <v>81</v>
       </c>
@@ -1675,7 +1669,7 @@
     </row>
     <row r="24" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="53"/>
-      <c r="B24" s="55"/>
+      <c r="B24" s="46"/>
       <c r="C24" s="39" t="s">
         <v>82</v>
       </c>
@@ -1694,9 +1688,9 @@
     </row>
     <row r="25" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="53"/>
-      <c r="B25" s="55"/>
+      <c r="B25" s="46"/>
       <c r="C25" s="39" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D25" s="17">
         <v>42</v>
@@ -1722,11 +1716,11 @@
     </row>
     <row r="27" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="53"/>
-      <c r="B27" s="56" t="s">
+      <c r="B27" s="47" t="s">
         <v>11</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D27" s="13">
         <v>19</v>
@@ -1743,9 +1737,9 @@
     </row>
     <row r="28" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="53"/>
-      <c r="B28" s="56"/>
+      <c r="B28" s="47"/>
       <c r="C28" s="9" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D28" s="13">
         <v>42</v>
@@ -1762,7 +1756,7 @@
     </row>
     <row r="29" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="53"/>
-      <c r="B29" s="56"/>
+      <c r="B29" s="47"/>
       <c r="C29" s="9" t="s">
         <v>40</v>
       </c>
@@ -1781,7 +1775,7 @@
     </row>
     <row r="30" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="53"/>
-      <c r="B30" s="56"/>
+      <c r="B30" s="47"/>
       <c r="C30" s="9" t="s">
         <v>41</v>
       </c>
@@ -1799,16 +1793,16 @@
       </c>
     </row>
     <row r="31" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="54"/>
-      <c r="B31" s="54"/>
-      <c r="C31" s="54"/>
-      <c r="D31" s="54"/>
-      <c r="E31" s="54"/>
-      <c r="F31" s="54"/>
-      <c r="G31" s="54"/>
+      <c r="A31" s="45"/>
+      <c r="B31" s="45"/>
+      <c r="C31" s="45"/>
+      <c r="D31" s="45"/>
+      <c r="E31" s="45"/>
+      <c r="F31" s="45"/>
+      <c r="G31" s="45"/>
     </row>
     <row r="32" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="57" t="s">
+      <c r="A32" s="51" t="s">
         <v>22</v>
       </c>
       <c r="B32" s="22" t="s">
@@ -1831,7 +1825,7 @@
       </c>
     </row>
     <row r="33" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="57"/>
+      <c r="A33" s="51"/>
       <c r="B33" s="22"/>
       <c r="C33" s="9" t="s">
         <v>92</v>
@@ -1850,7 +1844,7 @@
       </c>
     </row>
     <row r="34" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="57"/>
+      <c r="A34" s="51"/>
       <c r="B34" s="22"/>
       <c r="C34" s="9" t="s">
         <v>93</v>
@@ -1869,10 +1863,10 @@
       </c>
     </row>
     <row r="35" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="57"/>
+      <c r="A35" s="51"/>
       <c r="B35" s="22"/>
       <c r="C35" s="9" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D35" s="21">
         <v>42</v>
@@ -1888,7 +1882,7 @@
       </c>
     </row>
     <row r="36" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="57"/>
+      <c r="A36" s="51"/>
       <c r="B36" s="44"/>
       <c r="C36" s="44"/>
       <c r="D36" s="44"/>
@@ -1897,20 +1891,20 @@
       <c r="G36" s="44"/>
     </row>
     <row r="37" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="57"/>
+      <c r="A37" s="51"/>
       <c r="B37" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C37" s="48" t="s">
+      <c r="C37" s="54" t="s">
         <v>9</v>
       </c>
-      <c r="D37" s="49"/>
-      <c r="E37" s="49"/>
-      <c r="F37" s="50"/>
+      <c r="D37" s="55"/>
+      <c r="E37" s="55"/>
+      <c r="F37" s="56"/>
       <c r="G37" s="40"/>
     </row>
     <row r="38" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="57"/>
+      <c r="A38" s="51"/>
       <c r="B38" s="44"/>
       <c r="C38" s="44"/>
       <c r="D38" s="44"/>
@@ -1919,12 +1913,12 @@
       <c r="G38" s="44"/>
     </row>
     <row r="39" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="57"/>
+      <c r="A39" s="51"/>
       <c r="B39" s="22" t="s">
         <v>14</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D39" s="23">
         <v>20</v>
@@ -1933,17 +1927,17 @@
         <v>39</v>
       </c>
       <c r="F39" s="24" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G39" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="57"/>
+      <c r="A40" s="51"/>
       <c r="B40" s="25"/>
       <c r="C40" s="9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D40" s="23">
         <v>44</v>
@@ -1975,13 +1969,13 @@
         <v>7</v>
       </c>
       <c r="C42" s="11" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D42" s="13" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="F42" s="9" t="s">
         <v>77</v>
@@ -1994,10 +1988,10 @@
       <c r="A43" s="52"/>
       <c r="B43" s="22"/>
       <c r="C43" s="11" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="D43" s="13" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E43" s="11" t="s">
         <v>43</v>
@@ -2013,7 +2007,7 @@
       <c r="A44" s="52"/>
       <c r="B44" s="26"/>
       <c r="C44" s="11" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D44" s="13">
         <v>16</v>
@@ -2025,14 +2019,14 @@
         <v>87</v>
       </c>
       <c r="G44" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="52"/>
       <c r="B45" s="26"/>
       <c r="C45" s="9" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D45" s="13">
         <v>45</v>
@@ -2062,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D47" s="23">
         <v>21</v>
@@ -2081,7 +2075,7 @@
       <c r="A48" s="52"/>
       <c r="B48" s="27"/>
       <c r="C48" s="9" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D48" s="23">
         <v>50</v>
@@ -2100,7 +2094,7 @@
       <c r="A49" s="52"/>
       <c r="B49" s="27"/>
       <c r="C49" s="9" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D49" s="23">
         <v>25</v>
@@ -2109,10 +2103,10 @@
         <v>39</v>
       </c>
       <c r="F49" s="14" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G49" s="14" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
@@ -2129,13 +2123,13 @@
       <c r="B51" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="C51" s="51" t="s">
+      <c r="C51" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="D51" s="51"/>
-      <c r="E51" s="51"/>
-      <c r="F51" s="51"/>
-      <c r="G51" s="51"/>
+      <c r="D51" s="57"/>
+      <c r="E51" s="57"/>
+      <c r="F51" s="57"/>
+      <c r="G51" s="57"/>
     </row>
     <row r="52" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="52"/>
@@ -2151,22 +2145,22 @@
       <c r="B53" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="C53" s="51" t="s">
+      <c r="C53" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="D53" s="51"/>
-      <c r="E53" s="51"/>
-      <c r="F53" s="51"/>
-      <c r="G53" s="51"/>
+      <c r="D53" s="57"/>
+      <c r="E53" s="57"/>
+      <c r="F53" s="57"/>
+      <c r="G53" s="57"/>
     </row>
     <row r="54" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="54"/>
-      <c r="B54" s="54"/>
-      <c r="C54" s="54"/>
-      <c r="D54" s="54"/>
-      <c r="E54" s="54"/>
-      <c r="F54" s="54"/>
-      <c r="G54" s="54"/>
+      <c r="A54" s="45"/>
+      <c r="B54" s="45"/>
+      <c r="C54" s="45"/>
+      <c r="D54" s="45"/>
+      <c r="E54" s="45"/>
+      <c r="F54" s="45"/>
+      <c r="G54" s="45"/>
     </row>
     <row r="55" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="52" t="s">
@@ -2176,16 +2170,16 @@
         <v>16</v>
       </c>
       <c r="C55" s="9" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D55" s="17" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="E55" s="11" t="s">
         <v>29</v>
       </c>
       <c r="F55" s="14" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G55" s="18" t="s">
         <v>73</v>
@@ -2195,7 +2189,7 @@
       <c r="A56" s="52"/>
       <c r="B56" s="28"/>
       <c r="C56" s="43" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D56" s="17">
         <v>33</v>
@@ -2225,10 +2219,10 @@
         <v>15</v>
       </c>
       <c r="C58" s="11" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="D58" s="23" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E58" s="11" t="s">
         <v>30</v>
@@ -2244,10 +2238,10 @@
       <c r="A59" s="52"/>
       <c r="B59" s="30"/>
       <c r="C59" s="9" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D59" s="21" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E59" s="11" t="s">
         <v>47</v>
@@ -2320,7 +2314,7 @@
       <c r="A63" s="52"/>
       <c r="B63" s="30"/>
       <c r="C63" s="9" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D63" s="21">
         <v>32</v>
@@ -2339,7 +2333,7 @@
       <c r="A64" s="52"/>
       <c r="B64" s="30"/>
       <c r="C64" s="9" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D64" s="21">
         <v>31</v>
@@ -2348,17 +2342,17 @@
         <v>51</v>
       </c>
       <c r="F64" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G64" s="14" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="52"/>
       <c r="B65" s="30"/>
       <c r="C65" s="9" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D65" s="21">
         <v>45</v>
@@ -2370,14 +2364,14 @@
         <v>87</v>
       </c>
       <c r="G65" s="14" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="66" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="52"/>
       <c r="B66" s="30"/>
       <c r="C66" s="9" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D66" s="21">
         <v>34</v>
@@ -2396,7 +2390,7 @@
       <c r="A67" s="52"/>
       <c r="B67" s="30"/>
       <c r="C67" s="9" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D67" s="21">
         <v>17</v>
@@ -2415,13 +2409,13 @@
       <c r="A68" s="52"/>
       <c r="B68" s="30"/>
       <c r="C68" s="9" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D68" s="21">
         <v>52</v>
       </c>
       <c r="E68" s="11" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F68" s="9" t="s">
         <v>83</v>
@@ -2434,7 +2428,7 @@
       <c r="A69" s="52"/>
       <c r="B69" s="30"/>
       <c r="C69" s="9" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D69" s="21">
         <v>42</v>
@@ -2443,7 +2437,7 @@
         <v>42</v>
       </c>
       <c r="F69" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G69" s="14" t="s">
         <v>90</v>
@@ -2453,7 +2447,7 @@
       <c r="A70" s="52"/>
       <c r="B70" s="30"/>
       <c r="C70" s="9" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D70" s="21">
         <v>25</v>
@@ -2465,7 +2459,7 @@
         <v>75</v>
       </c>
       <c r="G70" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
@@ -2483,7 +2477,7 @@
         <v>14</v>
       </c>
       <c r="C72" s="9" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D72" s="17">
         <v>13</v>
@@ -2502,7 +2496,7 @@
       <c r="A73" s="52"/>
       <c r="B73" s="22"/>
       <c r="C73" s="11" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D73" s="23">
         <v>15</v>
@@ -2521,7 +2515,7 @@
       <c r="A74" s="52"/>
       <c r="B74" s="22"/>
       <c r="C74" s="11" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D74" s="23">
         <v>57</v>
@@ -2543,16 +2537,16 @@
         <v>55</v>
       </c>
       <c r="D75" s="23" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E75" s="11" t="s">
         <v>39</v>
       </c>
       <c r="F75" s="14" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G75" s="14" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="76" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
@@ -2570,7 +2564,7 @@
         <v>13</v>
       </c>
       <c r="C77" s="41" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D77" s="23">
         <v>33</v>
@@ -2579,17 +2573,17 @@
         <v>56</v>
       </c>
       <c r="F77" s="14" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G77" s="14" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="78" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="52"/>
       <c r="B78" s="32"/>
       <c r="C78" s="41" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D78" s="23">
         <v>45</v>
@@ -2598,10 +2592,10 @@
         <v>57</v>
       </c>
       <c r="F78" s="14" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G78" s="9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="79" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
@@ -2615,7 +2609,7 @@
     </row>
     <row r="80" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="52" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B80" s="22" t="s">
         <v>16</v>
@@ -2640,7 +2634,7 @@
       <c r="A81" s="52"/>
       <c r="B81" s="42"/>
       <c r="C81" s="18" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D81" s="17">
         <v>12</v>
@@ -2659,7 +2653,7 @@
       <c r="A82" s="52"/>
       <c r="B82" s="42"/>
       <c r="C82" s="18" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D82" s="17">
         <v>49</v>
@@ -2689,7 +2683,7 @@
         <v>15</v>
       </c>
       <c r="C84" s="18" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D84" s="13">
         <v>17</v>
@@ -2708,7 +2702,7 @@
       <c r="A85" s="52"/>
       <c r="B85" s="22"/>
       <c r="C85" s="14" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D85" s="13">
         <v>44</v>
@@ -2757,7 +2751,7 @@
       <c r="A88" s="52"/>
       <c r="B88" s="34"/>
       <c r="C88" s="9" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D88" s="21">
         <v>20</v>
@@ -2808,7 +2802,7 @@
       <c r="A91" s="53"/>
       <c r="B91" s="12"/>
       <c r="C91" s="9" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D91" s="23">
         <v>20</v>
@@ -2827,7 +2821,7 @@
       <c r="A92" s="53"/>
       <c r="B92" s="35"/>
       <c r="C92" s="18" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D92" s="23">
         <v>14</v>
@@ -2846,7 +2840,7 @@
       <c r="A93" s="53"/>
       <c r="B93" s="35"/>
       <c r="C93" s="9" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D93" s="23">
         <v>48</v>
@@ -2876,7 +2870,7 @@
         <v>11</v>
       </c>
       <c r="C95" s="11" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D95" s="23">
         <v>12</v>
@@ -2895,7 +2889,7 @@
       <c r="A96" s="53"/>
       <c r="B96" s="35"/>
       <c r="C96" s="11" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D96" s="23">
         <v>62</v>
@@ -2946,7 +2940,7 @@
       <c r="A99" s="52"/>
       <c r="B99" s="35"/>
       <c r="C99" s="9" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D99" s="17">
         <v>15</v>
@@ -2965,7 +2959,7 @@
       <c r="A100" s="52"/>
       <c r="B100" s="35"/>
       <c r="C100" s="11" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D100" s="23">
         <v>48</v>
@@ -2995,7 +2989,7 @@
         <v>15</v>
       </c>
       <c r="C102" s="9" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D102" s="23">
         <v>40</v>
@@ -3033,7 +3027,7 @@
       <c r="A104" s="52"/>
       <c r="B104" s="12"/>
       <c r="C104" s="9" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D104" s="23">
         <v>15</v>
@@ -3052,7 +3046,7 @@
       <c r="A105" s="52"/>
       <c r="B105" s="12"/>
       <c r="C105" s="11" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D105" s="23">
         <v>65</v>
@@ -3061,17 +3055,17 @@
         <v>63</v>
       </c>
       <c r="F105" s="14" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="G105" s="9" t="s">
-        <v>118</v>
+        <v>105</v>
       </c>
     </row>
     <row r="106" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A106" s="52"/>
       <c r="B106" s="12"/>
       <c r="C106" s="9" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D106" s="23">
         <v>22</v>
@@ -3093,7 +3087,7 @@
         <v>65</v>
       </c>
       <c r="D107" s="23" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E107" s="11" t="s">
         <v>32</v>
@@ -3119,13 +3113,13 @@
       <c r="B109" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C109" s="51" t="s">
+      <c r="C109" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="D109" s="51"/>
-      <c r="E109" s="51"/>
-      <c r="F109" s="51"/>
-      <c r="G109" s="51"/>
+      <c r="D109" s="57"/>
+      <c r="E109" s="57"/>
+      <c r="F109" s="57"/>
+      <c r="G109" s="57"/>
     </row>
     <row r="110" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="33"/>
@@ -3144,7 +3138,7 @@
         <v>19</v>
       </c>
       <c r="C111" s="9" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D111" s="13">
         <v>14</v>
@@ -3153,7 +3147,7 @@
         <v>32</v>
       </c>
       <c r="F111" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G111" s="9" t="s">
         <v>73</v>
@@ -3163,7 +3157,7 @@
       <c r="A112" s="52"/>
       <c r="B112" s="35"/>
       <c r="C112" s="9" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D112" s="13">
         <v>13</v>
@@ -3172,17 +3166,17 @@
         <v>35</v>
       </c>
       <c r="F112" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G112" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="113" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A113" s="52"/>
       <c r="B113" s="35"/>
       <c r="C113" s="11" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D113" s="13">
         <v>46</v>
@@ -3201,7 +3195,7 @@
       <c r="A114" s="52"/>
       <c r="B114" s="35"/>
       <c r="C114" s="11" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D114" s="13">
         <v>22</v>
@@ -3210,10 +3204,10 @@
         <v>31</v>
       </c>
       <c r="F114" s="14" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G114" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="115" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
@@ -3231,7 +3225,7 @@
         <v>10</v>
       </c>
       <c r="C116" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D116" s="13">
         <v>16</v>
@@ -3240,17 +3234,17 @@
         <v>32</v>
       </c>
       <c r="F116" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G116" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="117" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A117" s="52"/>
       <c r="B117" s="35"/>
       <c r="C117" s="9" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D117" s="13">
         <v>33</v>
@@ -3259,17 +3253,17 @@
         <v>35</v>
       </c>
       <c r="F117" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G117" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="118" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A118" s="52"/>
       <c r="B118" s="35"/>
       <c r="C118" s="9" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D118" s="13">
         <v>19</v>
@@ -3278,7 +3272,7 @@
         <v>38</v>
       </c>
       <c r="F118" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G118" s="9" t="s">
         <v>83</v>
@@ -3298,13 +3292,13 @@
       <c r="B120" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="C120" s="51" t="s">
+      <c r="C120" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="D120" s="51"/>
-      <c r="E120" s="51"/>
-      <c r="F120" s="51"/>
-      <c r="G120" s="51"/>
+      <c r="D120" s="57"/>
+      <c r="E120" s="57"/>
+      <c r="F120" s="57"/>
+      <c r="G120" s="57"/>
     </row>
     <row r="121" spans="1:7" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A121" s="52"/>
@@ -3321,7 +3315,7 @@
         <v>12</v>
       </c>
       <c r="C122" s="41" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D122" s="13">
         <v>41</v>
@@ -3330,10 +3324,10 @@
         <v>69</v>
       </c>
       <c r="F122" s="14" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G122" s="14" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="123" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3350,29 +3344,29 @@
         <v>28</v>
       </c>
       <c r="B124" s="35" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C124" s="9" t="s">
         <v>67</v>
       </c>
       <c r="D124" s="13" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E124" s="11" t="s">
         <v>29</v>
       </c>
       <c r="F124" s="14" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G124" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="125" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A125" s="52"/>
       <c r="B125" s="35"/>
       <c r="C125" s="9" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D125" s="13">
         <v>15</v>
@@ -3391,7 +3385,7 @@
       <c r="A126" s="52"/>
       <c r="B126" s="35"/>
       <c r="C126" s="9" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D126" s="13">
         <v>59</v>
@@ -3413,7 +3407,7 @@
         <v>68</v>
       </c>
       <c r="D127" s="13" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E127" s="11" t="s">
         <v>31</v>
@@ -3429,32 +3423,32 @@
       <c r="A128" s="52"/>
       <c r="B128" s="35"/>
       <c r="C128" s="9" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D128" s="13" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="E128" s="11" t="s">
         <v>32</v>
       </c>
       <c r="F128" s="14" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="G128" s="9" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="129" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A129" s="52"/>
       <c r="B129" s="35"/>
       <c r="C129" s="9" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D129" s="13">
         <v>34</v>
       </c>
       <c r="E129" s="11" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F129" s="14" t="s">
         <v>75</v>
@@ -3474,21 +3468,22 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="B108:G108"/>
-    <mergeCell ref="B15:G15"/>
-    <mergeCell ref="A20:G20"/>
-    <mergeCell ref="B11:G11"/>
-    <mergeCell ref="B52:G52"/>
-    <mergeCell ref="B79:G79"/>
-    <mergeCell ref="B57:G57"/>
-    <mergeCell ref="A54:G54"/>
-    <mergeCell ref="B22:B25"/>
-    <mergeCell ref="B27:B30"/>
-    <mergeCell ref="C21:F21"/>
-    <mergeCell ref="B26:G26"/>
-    <mergeCell ref="A32:A40"/>
-    <mergeCell ref="A80:A88"/>
-    <mergeCell ref="A90:A96"/>
+    <mergeCell ref="C110:G110"/>
+    <mergeCell ref="C9:F9"/>
+    <mergeCell ref="C37:F37"/>
+    <mergeCell ref="C121:G121"/>
+    <mergeCell ref="C109:G109"/>
+    <mergeCell ref="C120:G120"/>
+    <mergeCell ref="C51:G51"/>
+    <mergeCell ref="C53:G53"/>
+    <mergeCell ref="B101:G101"/>
+    <mergeCell ref="C115:G115"/>
+    <mergeCell ref="B71:G71"/>
+    <mergeCell ref="A89:G89"/>
+    <mergeCell ref="B86:G86"/>
+    <mergeCell ref="B83:G83"/>
+    <mergeCell ref="B76:F76"/>
+    <mergeCell ref="A98:A109"/>
     <mergeCell ref="A124:A130"/>
     <mergeCell ref="C130:G130"/>
     <mergeCell ref="A111:A122"/>
@@ -3505,22 +3500,21 @@
     <mergeCell ref="A31:G31"/>
     <mergeCell ref="C119:G119"/>
     <mergeCell ref="B94:G94"/>
-    <mergeCell ref="C110:G110"/>
-    <mergeCell ref="C9:F9"/>
-    <mergeCell ref="C37:F37"/>
-    <mergeCell ref="C121:G121"/>
-    <mergeCell ref="C109:G109"/>
-    <mergeCell ref="C120:G120"/>
-    <mergeCell ref="C51:G51"/>
-    <mergeCell ref="C53:G53"/>
-    <mergeCell ref="B101:G101"/>
-    <mergeCell ref="C115:G115"/>
-    <mergeCell ref="B71:G71"/>
-    <mergeCell ref="A89:G89"/>
-    <mergeCell ref="B86:G86"/>
-    <mergeCell ref="B83:G83"/>
-    <mergeCell ref="B76:F76"/>
-    <mergeCell ref="A98:A109"/>
+    <mergeCell ref="B108:G108"/>
+    <mergeCell ref="B15:G15"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="B11:G11"/>
+    <mergeCell ref="B52:G52"/>
+    <mergeCell ref="B79:G79"/>
+    <mergeCell ref="B57:G57"/>
+    <mergeCell ref="A54:G54"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="B27:B30"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="B26:G26"/>
+    <mergeCell ref="A32:A40"/>
+    <mergeCell ref="A80:A88"/>
+    <mergeCell ref="A90:A96"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.625" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="53" fitToHeight="0" orientation="portrait" r:id="rId1"/>

</xml_diff>